<commit_message>
feat: add SEO keywords and structured data support
- Introduced a new file `deliverables/seo_keywords.txt` containing relevant SEO keywords in Persian and English.
- Created a `docs/dev-journal/JOURNAL.md` to maintain an append-only record of codebase changes and decisions.
- Implemented JSON-LD builders in `src/lib/structured-data.ts` for structured data across the site, including organization, website, breadcrumb, and product schemas.
- Enhanced technical SEO by integrating structured data into various pages, ensuring compliance with existing plans and avoiding fabricated claims.
</commit_message>
<xml_diff>
--- a/deliverables/Elecio_SEO_Content_Planner_FA.xlsx
+++ b/deliverables/Elecio_SEO_Content_Planner_FA.xlsx
@@ -26,8 +26,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -140,7 +140,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -162,12 +162,56 @@
         <color rgb="00D7E0EC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D7E0EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D7E0EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7E0EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D7E0EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D7E0EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D7E0EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7E0EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D7E0EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -200,7 +244,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -209,10 +253,10 @@
     <xf numFmtId="9" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -221,7 +265,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,6 +277,26 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -394,7 +458,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -968,12 +1031,12 @@
           <t>در «نقشه کیورد»، حجم جست‌وجو، سختی، رتبه، کلیک و ایمپرشن را فقط از Google Search Console، Keyword Planner یا ابزار معتبر وارد کنید.</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="28" t="n"/>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -986,12 +1049,12 @@
           <t>ابتدا موضوعات با نیت تجاری، ارتباط مستقیم با محصول و شکاف محتوایی واقعی را انتخاب کنید. داشبورد وضعیت را خلاصه می‌کند.</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="28" t="n"/>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1004,12 +1067,12 @@
           <t>در «بریف مقاله» شناسه‌ای مثل EC-006 را انتخاب کنید؛ عنوان، کیورد، متا، ساختار و لینک‌ها خودکار نمایش داده می‌شوند. خانه‌های زرد را تیم فنی/سئو تکمیل کند.</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="28" t="n"/>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1022,12 +1085,12 @@
           <t>پرامپت اختصاصی را با داده‌های بریف کامل کنید. در موضوعات فنی، کاتالوگ و تأیید تیم محصول باید بر متن AI مقدم باشد.</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="28" t="n"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1040,12 +1103,12 @@
           <t>قبل از انتشار تمام موارد وزن ۵ در چک‌لیست باید تأیید شوند. سپس نگارش، موبایل، لینک‌ها و متادیتا بررسی شود.</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="28" t="n"/>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1058,12 +1121,12 @@
           <t>هر مقاله به صفحه Pillar مرتبط و دو مقاله هم‌خوشه لینک بدهد. انکر را طبیعی و متنوع انتخاب کنید.</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="27" t="n"/>
+      <c r="E9" s="27" t="n"/>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="28" t="n"/>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -1076,12 +1139,12 @@
           <t>لینک انتشار، وضعیت، درصد پیشرفت و تاریخ به‌روزرسانی را ثبت کنید؛ پس از ۲۸ تا ۴۲ روز داده GSC را بررسی و محتوا را بهبود دهید.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="28" t="n"/>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1094,12 +1157,12 @@
           <t>این فایل پیشنهاد استراتژیک است، نه داده تحقیق کیورد. حجم و رتبه تخمینی ساخته نشده و باید با داده واقعی بازار ایران تکمیل شود.</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="27" t="n"/>
+      <c r="E11" s="27" t="n"/>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1163,12 +1226,12 @@
           <t>تو یک نویسنده متخصص سئوی فارسی، استراتژیست محتوای B2B صنعتی و آشنا با CNC، DNC، کنترلرهای FANUC، Siemens، Heidenhain و ارتباط RS232/شبکه هستی.</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="28" t="n"/>
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
@@ -1187,12 +1250,12 @@
 منابع تأییدشده: {{منابع}}</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="28" t="n"/>
     </row>
     <row r="6" ht="70" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
@@ -1205,12 +1268,12 @@
           <t>یک مقاله فارسی کامل، کاربردی و قابل انتشار برای وب‌سایت ElecIO بنویس که مسئله واقعی مدیر کارگاه، برنامه‌نویس یا اپراتور CNC را حل کند. انسان‌محور بنویس و از Keyword Stuffing پرهیز کن.</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="28" t="n"/>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -1223,12 +1286,12 @@
           <t>هیچ آمار، قیمت، قانون، استاندارد، سازگاری کنترلر یا مشخصه فنی را اختراع نکن. برای مشخصات ElecIO فقط از کاتالوگ رسمی، صفحات محصول و اطلاعات تأییدشده استفاده کن. اگر داده‌ای موجود نیست، شفاف بگو نیازمند تأیید فنی است.</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="28" t="n"/>
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -1241,12 +1304,12 @@
           <t>حداقل ۱۵۰۰ واژه مفید و کاملاً فارسی. اصطلاحات انگلیسی تخصصی را در صورت نیاز کنار معادل فارسی بیاور. از لحن رباتیک، مقدمه طولانی و تکرار مصنوعی خودداری کن.</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="28" t="n"/>
     </row>
     <row r="9" ht="70" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
@@ -1259,12 +1322,12 @@
           <t>یک H1 قوی، مقدمه کوتاه، H2های قابل جست‌وجو، H3 برای مراحل/مثال‌ها/اشتباهات، حداقل یک جدول مفید در صورت نیاز، مثال عملی کارگاهی، نکات اجرایی، FAQ واقعی و جمع‌بندی تصمیم‌ساز.</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="27" t="n"/>
+      <c r="E9" s="27" t="n"/>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="28" t="n"/>
     </row>
     <row r="10" ht="70" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -1277,12 +1340,12 @@
           <t>در ابتدای خروجی این موارد را بده: SEO Title، Meta Description، Slug انگلیسی پیشنهادی، Focus Keyword، Secondary Keywords، دسته پیشنهادی، برچسب‌های محدود و مرتبط.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="28" t="n"/>
     </row>
     <row r="11" ht="70" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
@@ -1295,12 +1358,12 @@
           <t>لینک داخلی را با قالب [پیشنهاد لینک داخلی: انکر — URL] و فقط در جای طبیعی پیشنهاد بده. حداقل یک لینک به Pillar مرتبط و دو لینک به مقالات هم‌خوشه. لینک خارجی فقط به منابع رسمی و معتبر، در صورت ارزش واقعی.</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="27" t="n"/>
+      <c r="E11" s="27" t="n"/>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
+      <c r="H11" s="28" t="n"/>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
@@ -1313,12 +1376,12 @@
           <t>تصویر نساز، Placeholder تصویر، محل تصویر، کپشن یا Alt Text پیشنهاد نده.</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="C12" s="27" t="n"/>
+      <c r="D12" s="27" t="n"/>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="28" t="n"/>
     </row>
     <row r="13" ht="70" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
@@ -1331,12 +1394,12 @@
           <t>در صورت درخواست فایل Word: بدون Header و Footer، با Heading Style صحیح، فاصله خطوط ۲.۲، پاراگراف‌های خوانا، فهرست‌های استاندارد و جدول‌های حرفه‌ای تحویل بده.</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="28" t="n"/>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
@@ -1349,12 +1412,12 @@
           <t>پیش از تحویل بررسی کن: حداقل ۱۵۰۰ واژه، پاسخ کامل به نیت، ساختار درست، استفاده طبیعی کیورد، منابع قابل اتکا، FAQ، جمع‌بندی، لینک داخلی، CTA و نبود ادعای ساختگی.</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="28" t="n"/>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -1374,12 +1437,12 @@
 ۸) لینک‌های داخلی و خارجی پیشنهادی</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="27" t="n"/>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -6931,7 +6994,7 @@
       </c>
       <c r="V4" s="12" t="inlineStr"/>
       <c r="W4" s="12" t="inlineStr"/>
-      <c r="X4" s="14" t="n">
+      <c r="X4" s="29" t="n">
         <v>46249</v>
       </c>
       <c r="Y4" s="15" t="inlineStr">
@@ -6952,10 +7015,14 @@
       <c r="AB4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="AC4" s="17" t="n">
+      <c r="AC4" s="30" t="n">
         <v>46247</v>
       </c>
-      <c r="AD4" s="12" t="inlineStr"/>
+      <c r="AD4" s="12" t="inlineStr">
+        <is>
+          <t>مقاله کامل و عمیق (حدود 3800 کلمه)، اسکیما TechArticle+FAQPage.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="72" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
@@ -7068,7 +7135,7 @@
       </c>
       <c r="V5" s="13" t="inlineStr"/>
       <c r="W5" s="13" t="inlineStr"/>
-      <c r="X5" s="18" t="n">
+      <c r="X5" s="31" t="n">
         <v>46250</v>
       </c>
       <c r="Y5" s="19" t="inlineStr">
@@ -7089,10 +7156,14 @@
       <c r="AB5" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="AC5" s="21" t="n">
+      <c r="AC5" s="32" t="n">
         <v>46247</v>
       </c>
-      <c r="AD5" s="13" t="inlineStr"/>
+      <c r="AD5" s="13" t="inlineStr">
+        <is>
+          <t>منتشرشده اما کوتاه (حدود 140 کلمه)، فاقد Focus Keyword ثبت‌شده. نیازمند Expand طبق بخش 5 برنامه قبل از ارتقای Schema.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="72" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
@@ -7205,7 +7276,7 @@
       </c>
       <c r="V6" s="12" t="inlineStr"/>
       <c r="W6" s="12" t="inlineStr"/>
-      <c r="X6" s="14" t="n">
+      <c r="X6" s="29" t="n">
         <v>46251</v>
       </c>
       <c r="Y6" s="15" t="inlineStr">
@@ -7226,10 +7297,14 @@
       <c r="AB6" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="AC6" s="17" t="n">
+      <c r="AC6" s="30" t="n">
         <v>46247</v>
       </c>
-      <c r="AD6" s="12" t="inlineStr"/>
+      <c r="AD6" s="12" t="inlineStr">
+        <is>
+          <t>منتشرشده اما کوتاه (حدود 140 کلمه)، فاقد Focus Keyword ثبت‌شده. نیازمند Expand.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
@@ -7342,7 +7417,7 @@
       </c>
       <c r="V7" s="13" t="inlineStr"/>
       <c r="W7" s="13" t="inlineStr"/>
-      <c r="X7" s="18" t="n">
+      <c r="X7" s="31" t="n">
         <v>46252</v>
       </c>
       <c r="Y7" s="19" t="inlineStr">
@@ -7363,10 +7438,14 @@
       <c r="AB7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="AC7" s="21" t="n">
+      <c r="AC7" s="32" t="n">
         <v>46247</v>
       </c>
-      <c r="AD7" s="13" t="inlineStr"/>
+      <c r="AD7" s="13" t="inlineStr">
+        <is>
+          <t>منتشرشده اما کوتاه (حدود 140 کلمه)، فاقد Focus Keyword ثبت‌شده. نیازمند Expand.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
@@ -7479,7 +7558,7 @@
       </c>
       <c r="V8" s="12" t="inlineStr"/>
       <c r="W8" s="12" t="inlineStr"/>
-      <c r="X8" s="14" t="n">
+      <c r="X8" s="29" t="n">
         <v>46253</v>
       </c>
       <c r="Y8" s="15" t="inlineStr">
@@ -7500,10 +7579,14 @@
       <c r="AB8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="AC8" s="17" t="n">
+      <c r="AC8" s="30" t="n">
         <v>46247</v>
       </c>
-      <c r="AD8" s="12" t="inlineStr"/>
+      <c r="AD8" s="12" t="inlineStr">
+        <is>
+          <t>منتشرشده اما کوتاه (حدود 140 کلمه)، فاقد Focus Keyword ثبت‌شده. نیازمند Expand.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
@@ -7616,7 +7699,7 @@
       </c>
       <c r="V9" s="13" t="inlineStr"/>
       <c r="W9" s="13" t="inlineStr"/>
-      <c r="X9" s="18" t="n">
+      <c r="X9" s="31" t="n">
         <v>46256</v>
       </c>
       <c r="Y9" s="13" t="inlineStr"/>
@@ -7747,7 +7830,7 @@
       </c>
       <c r="V10" s="12" t="inlineStr"/>
       <c r="W10" s="12" t="inlineStr"/>
-      <c r="X10" s="14" t="n">
+      <c r="X10" s="29" t="n">
         <v>46257</v>
       </c>
       <c r="Y10" s="12" t="inlineStr"/>
@@ -7878,7 +7961,7 @@
       </c>
       <c r="V11" s="13" t="inlineStr"/>
       <c r="W11" s="13" t="inlineStr"/>
-      <c r="X11" s="18" t="n">
+      <c r="X11" s="31" t="n">
         <v>46258</v>
       </c>
       <c r="Y11" s="13" t="inlineStr"/>
@@ -8009,7 +8092,7 @@
       </c>
       <c r="V12" s="12" t="inlineStr"/>
       <c r="W12" s="12" t="inlineStr"/>
-      <c r="X12" s="14" t="n">
+      <c r="X12" s="29" t="n">
         <v>46259</v>
       </c>
       <c r="Y12" s="12" t="inlineStr"/>
@@ -8140,7 +8223,7 @@
       </c>
       <c r="V13" s="13" t="inlineStr"/>
       <c r="W13" s="13" t="inlineStr"/>
-      <c r="X13" s="18" t="n">
+      <c r="X13" s="31" t="n">
         <v>46260</v>
       </c>
       <c r="Y13" s="13" t="inlineStr"/>
@@ -8271,7 +8354,7 @@
       </c>
       <c r="V14" s="12" t="inlineStr"/>
       <c r="W14" s="12" t="inlineStr"/>
-      <c r="X14" s="14" t="n">
+      <c r="X14" s="29" t="n">
         <v>46263</v>
       </c>
       <c r="Y14" s="12" t="inlineStr"/>
@@ -8402,7 +8485,7 @@
       </c>
       <c r="V15" s="13" t="inlineStr"/>
       <c r="W15" s="13" t="inlineStr"/>
-      <c r="X15" s="18" t="n">
+      <c r="X15" s="31" t="n">
         <v>46264</v>
       </c>
       <c r="Y15" s="13" t="inlineStr"/>
@@ -8533,7 +8616,7 @@
       </c>
       <c r="V16" s="12" t="inlineStr"/>
       <c r="W16" s="12" t="inlineStr"/>
-      <c r="X16" s="14" t="n">
+      <c r="X16" s="29" t="n">
         <v>46265</v>
       </c>
       <c r="Y16" s="12" t="inlineStr"/>
@@ -8664,7 +8747,7 @@
       </c>
       <c r="V17" s="13" t="inlineStr"/>
       <c r="W17" s="13" t="inlineStr"/>
-      <c r="X17" s="18" t="n">
+      <c r="X17" s="31" t="n">
         <v>46266</v>
       </c>
       <c r="Y17" s="13" t="inlineStr"/>
@@ -8795,7 +8878,7 @@
       </c>
       <c r="V18" s="12" t="inlineStr"/>
       <c r="W18" s="12" t="inlineStr"/>
-      <c r="X18" s="14" t="n">
+      <c r="X18" s="29" t="n">
         <v>46267</v>
       </c>
       <c r="Y18" s="12" t="inlineStr"/>
@@ -8926,7 +9009,7 @@
       </c>
       <c r="V19" s="13" t="inlineStr"/>
       <c r="W19" s="13" t="inlineStr"/>
-      <c r="X19" s="18" t="n">
+      <c r="X19" s="31" t="n">
         <v>46270</v>
       </c>
       <c r="Y19" s="13" t="inlineStr"/>
@@ -9057,7 +9140,7 @@
       </c>
       <c r="V20" s="12" t="inlineStr"/>
       <c r="W20" s="12" t="inlineStr"/>
-      <c r="X20" s="14" t="n">
+      <c r="X20" s="29" t="n">
         <v>46271</v>
       </c>
       <c r="Y20" s="12" t="inlineStr"/>
@@ -9188,7 +9271,7 @@
       </c>
       <c r="V21" s="13" t="inlineStr"/>
       <c r="W21" s="13" t="inlineStr"/>
-      <c r="X21" s="18" t="n">
+      <c r="X21" s="31" t="n">
         <v>46272</v>
       </c>
       <c r="Y21" s="13" t="inlineStr"/>
@@ -9319,7 +9402,7 @@
       </c>
       <c r="V22" s="12" t="inlineStr"/>
       <c r="W22" s="12" t="inlineStr"/>
-      <c r="X22" s="14" t="n">
+      <c r="X22" s="29" t="n">
         <v>46273</v>
       </c>
       <c r="Y22" s="12" t="inlineStr"/>
@@ -9450,7 +9533,7 @@
       </c>
       <c r="V23" s="13" t="inlineStr"/>
       <c r="W23" s="13" t="inlineStr"/>
-      <c r="X23" s="18" t="n">
+      <c r="X23" s="31" t="n">
         <v>46274</v>
       </c>
       <c r="Y23" s="13" t="inlineStr"/>
@@ -9581,7 +9664,7 @@
       </c>
       <c r="V24" s="12" t="inlineStr"/>
       <c r="W24" s="12" t="inlineStr"/>
-      <c r="X24" s="14" t="n">
+      <c r="X24" s="29" t="n">
         <v>46277</v>
       </c>
       <c r="Y24" s="12" t="inlineStr"/>
@@ -9712,7 +9795,7 @@
       </c>
       <c r="V25" s="13" t="inlineStr"/>
       <c r="W25" s="13" t="inlineStr"/>
-      <c r="X25" s="18" t="n">
+      <c r="X25" s="31" t="n">
         <v>46278</v>
       </c>
       <c r="Y25" s="13" t="inlineStr"/>
@@ -9843,7 +9926,7 @@
       </c>
       <c r="V26" s="12" t="inlineStr"/>
       <c r="W26" s="12" t="inlineStr"/>
-      <c r="X26" s="14" t="n">
+      <c r="X26" s="29" t="n">
         <v>46279</v>
       </c>
       <c r="Y26" s="12" t="inlineStr"/>
@@ -9974,7 +10057,7 @@
       </c>
       <c r="V27" s="13" t="inlineStr"/>
       <c r="W27" s="13" t="inlineStr"/>
-      <c r="X27" s="18" t="n">
+      <c r="X27" s="31" t="n">
         <v>46280</v>
       </c>
       <c r="Y27" s="13" t="inlineStr"/>
@@ -10105,7 +10188,7 @@
       </c>
       <c r="V28" s="12" t="inlineStr"/>
       <c r="W28" s="12" t="inlineStr"/>
-      <c r="X28" s="14" t="n">
+      <c r="X28" s="29" t="n">
         <v>46281</v>
       </c>
       <c r="Y28" s="12" t="inlineStr"/>
@@ -10236,7 +10319,7 @@
       </c>
       <c r="V29" s="13" t="inlineStr"/>
       <c r="W29" s="13" t="inlineStr"/>
-      <c r="X29" s="18" t="n">
+      <c r="X29" s="31" t="n">
         <v>46284</v>
       </c>
       <c r="Y29" s="13" t="inlineStr"/>
@@ -10367,7 +10450,7 @@
       </c>
       <c r="V30" s="12" t="inlineStr"/>
       <c r="W30" s="12" t="inlineStr"/>
-      <c r="X30" s="14" t="n">
+      <c r="X30" s="29" t="n">
         <v>46285</v>
       </c>
       <c r="Y30" s="12" t="inlineStr"/>
@@ -10498,7 +10581,7 @@
       </c>
       <c r="V31" s="13" t="inlineStr"/>
       <c r="W31" s="13" t="inlineStr"/>
-      <c r="X31" s="18" t="n">
+      <c r="X31" s="31" t="n">
         <v>46286</v>
       </c>
       <c r="Y31" s="13" t="inlineStr"/>
@@ -10629,7 +10712,7 @@
       </c>
       <c r="V32" s="12" t="inlineStr"/>
       <c r="W32" s="12" t="inlineStr"/>
-      <c r="X32" s="14" t="n">
+      <c r="X32" s="29" t="n">
         <v>46287</v>
       </c>
       <c r="Y32" s="12" t="inlineStr"/>
@@ -10760,7 +10843,7 @@
       </c>
       <c r="V33" s="13" t="inlineStr"/>
       <c r="W33" s="13" t="inlineStr"/>
-      <c r="X33" s="18" t="n">
+      <c r="X33" s="31" t="n">
         <v>46288</v>
       </c>
       <c r="Y33" s="13" t="inlineStr"/>
@@ -10891,7 +10974,7 @@
       </c>
       <c r="V34" s="12" t="inlineStr"/>
       <c r="W34" s="12" t="inlineStr"/>
-      <c r="X34" s="14" t="n">
+      <c r="X34" s="29" t="n">
         <v>46291</v>
       </c>
       <c r="Y34" s="12" t="inlineStr"/>
@@ -11022,7 +11105,7 @@
       </c>
       <c r="V35" s="13" t="inlineStr"/>
       <c r="W35" s="13" t="inlineStr"/>
-      <c r="X35" s="18" t="n">
+      <c r="X35" s="31" t="n">
         <v>46292</v>
       </c>
       <c r="Y35" s="13" t="inlineStr"/>
@@ -11153,7 +11236,7 @@
       </c>
       <c r="V36" s="12" t="inlineStr"/>
       <c r="W36" s="12" t="inlineStr"/>
-      <c r="X36" s="14" t="n">
+      <c r="X36" s="29" t="n">
         <v>46293</v>
       </c>
       <c r="Y36" s="12" t="inlineStr"/>
@@ -11284,7 +11367,7 @@
       </c>
       <c r="V37" s="13" t="inlineStr"/>
       <c r="W37" s="13" t="inlineStr"/>
-      <c r="X37" s="18" t="n">
+      <c r="X37" s="31" t="n">
         <v>46294</v>
       </c>
       <c r="Y37" s="13" t="inlineStr"/>
@@ -11415,7 +11498,7 @@
       </c>
       <c r="V38" s="12" t="inlineStr"/>
       <c r="W38" s="12" t="inlineStr"/>
-      <c r="X38" s="14" t="n">
+      <c r="X38" s="29" t="n">
         <v>46295</v>
       </c>
       <c r="Y38" s="12" t="inlineStr"/>
@@ -11546,7 +11629,7 @@
       </c>
       <c r="V39" s="13" t="inlineStr"/>
       <c r="W39" s="13" t="inlineStr"/>
-      <c r="X39" s="18" t="n">
+      <c r="X39" s="31" t="n">
         <v>46298</v>
       </c>
       <c r="Y39" s="13" t="inlineStr"/>
@@ -11677,7 +11760,7 @@
       </c>
       <c r="V40" s="12" t="inlineStr"/>
       <c r="W40" s="12" t="inlineStr"/>
-      <c r="X40" s="14" t="n">
+      <c r="X40" s="29" t="n">
         <v>46299</v>
       </c>
       <c r="Y40" s="12" t="inlineStr"/>
@@ -11808,7 +11891,7 @@
       </c>
       <c r="V41" s="13" t="inlineStr"/>
       <c r="W41" s="13" t="inlineStr"/>
-      <c r="X41" s="18" t="n">
+      <c r="X41" s="31" t="n">
         <v>46300</v>
       </c>
       <c r="Y41" s="13" t="inlineStr"/>
@@ -11939,7 +12022,7 @@
       </c>
       <c r="V42" s="12" t="inlineStr"/>
       <c r="W42" s="12" t="inlineStr"/>
-      <c r="X42" s="14" t="n">
+      <c r="X42" s="29" t="n">
         <v>46301</v>
       </c>
       <c r="Y42" s="12" t="inlineStr"/>
@@ -12070,7 +12153,7 @@
       </c>
       <c r="V43" s="13" t="inlineStr"/>
       <c r="W43" s="13" t="inlineStr"/>
-      <c r="X43" s="18" t="n">
+      <c r="X43" s="31" t="n">
         <v>46302</v>
       </c>
       <c r="Y43" s="13" t="inlineStr"/>
@@ -12201,7 +12284,7 @@
       </c>
       <c r="V44" s="12" t="inlineStr"/>
       <c r="W44" s="12" t="inlineStr"/>
-      <c r="X44" s="14" t="n">
+      <c r="X44" s="29" t="n">
         <v>46305</v>
       </c>
       <c r="Y44" s="12" t="inlineStr"/>
@@ -12332,7 +12415,7 @@
       </c>
       <c r="V45" s="13" t="inlineStr"/>
       <c r="W45" s="13" t="inlineStr"/>
-      <c r="X45" s="18" t="n">
+      <c r="X45" s="31" t="n">
         <v>46306</v>
       </c>
       <c r="Y45" s="13" t="inlineStr"/>
@@ -12463,7 +12546,7 @@
       </c>
       <c r="V46" s="12" t="inlineStr"/>
       <c r="W46" s="12" t="inlineStr"/>
-      <c r="X46" s="14" t="n">
+      <c r="X46" s="29" t="n">
         <v>46307</v>
       </c>
       <c r="Y46" s="12" t="inlineStr"/>
@@ -12594,7 +12677,7 @@
       </c>
       <c r="V47" s="13" t="inlineStr"/>
       <c r="W47" s="13" t="inlineStr"/>
-      <c r="X47" s="18" t="n">
+      <c r="X47" s="31" t="n">
         <v>46308</v>
       </c>
       <c r="Y47" s="13" t="inlineStr"/>
@@ -12725,7 +12808,7 @@
       </c>
       <c r="V48" s="12" t="inlineStr"/>
       <c r="W48" s="12" t="inlineStr"/>
-      <c r="X48" s="14" t="n">
+      <c r="X48" s="29" t="n">
         <v>46309</v>
       </c>
       <c r="Y48" s="12" t="inlineStr"/>
@@ -12856,7 +12939,7 @@
       </c>
       <c r="V49" s="13" t="inlineStr"/>
       <c r="W49" s="13" t="inlineStr"/>
-      <c r="X49" s="18" t="n">
+      <c r="X49" s="31" t="n">
         <v>46312</v>
       </c>
       <c r="Y49" s="13" t="inlineStr"/>
@@ -12987,7 +13070,7 @@
       </c>
       <c r="V50" s="12" t="inlineStr"/>
       <c r="W50" s="12" t="inlineStr"/>
-      <c r="X50" s="14" t="n">
+      <c r="X50" s="29" t="n">
         <v>46313</v>
       </c>
       <c r="Y50" s="12" t="inlineStr"/>
@@ -13118,7 +13201,7 @@
       </c>
       <c r="V51" s="13" t="inlineStr"/>
       <c r="W51" s="13" t="inlineStr"/>
-      <c r="X51" s="18" t="n">
+      <c r="X51" s="31" t="n">
         <v>46314</v>
       </c>
       <c r="Y51" s="13" t="inlineStr"/>
@@ -13249,7 +13332,7 @@
       </c>
       <c r="V52" s="12" t="inlineStr"/>
       <c r="W52" s="12" t="inlineStr"/>
-      <c r="X52" s="14" t="n">
+      <c r="X52" s="29" t="n">
         <v>46315</v>
       </c>
       <c r="Y52" s="12" t="inlineStr"/>
@@ -13380,7 +13463,7 @@
       </c>
       <c r="V53" s="13" t="inlineStr"/>
       <c r="W53" s="13" t="inlineStr"/>
-      <c r="X53" s="18" t="n">
+      <c r="X53" s="31" t="n">
         <v>46316</v>
       </c>
       <c r="Y53" s="13" t="inlineStr"/>
@@ -13511,7 +13594,7 @@
       </c>
       <c r="V54" s="12" t="inlineStr"/>
       <c r="W54" s="12" t="inlineStr"/>
-      <c r="X54" s="14" t="n">
+      <c r="X54" s="29" t="n">
         <v>46319</v>
       </c>
       <c r="Y54" s="12" t="inlineStr"/>
@@ -13642,7 +13725,7 @@
       </c>
       <c r="V55" s="13" t="inlineStr"/>
       <c r="W55" s="13" t="inlineStr"/>
-      <c r="X55" s="18" t="n">
+      <c r="X55" s="31" t="n">
         <v>46320</v>
       </c>
       <c r="Y55" s="13" t="inlineStr"/>
@@ -13773,7 +13856,7 @@
       </c>
       <c r="V56" s="12" t="inlineStr"/>
       <c r="W56" s="12" t="inlineStr"/>
-      <c r="X56" s="14" t="n">
+      <c r="X56" s="29" t="n">
         <v>46321</v>
       </c>
       <c r="Y56" s="12" t="inlineStr"/>
@@ -13904,7 +13987,7 @@
       </c>
       <c r="V57" s="13" t="inlineStr"/>
       <c r="W57" s="13" t="inlineStr"/>
-      <c r="X57" s="18" t="n">
+      <c r="X57" s="31" t="n">
         <v>46322</v>
       </c>
       <c r="Y57" s="13" t="inlineStr"/>
@@ -14035,7 +14118,7 @@
       </c>
       <c r="V58" s="12" t="inlineStr"/>
       <c r="W58" s="12" t="inlineStr"/>
-      <c r="X58" s="14" t="n">
+      <c r="X58" s="29" t="n">
         <v>46323</v>
       </c>
       <c r="Y58" s="12" t="inlineStr"/>
@@ -14166,7 +14249,7 @@
       </c>
       <c r="V59" s="13" t="inlineStr"/>
       <c r="W59" s="13" t="inlineStr"/>
-      <c r="X59" s="18" t="n">
+      <c r="X59" s="31" t="n">
         <v>46326</v>
       </c>
       <c r="Y59" s="13" t="inlineStr"/>
@@ -14297,7 +14380,7 @@
       </c>
       <c r="V60" s="12" t="inlineStr"/>
       <c r="W60" s="12" t="inlineStr"/>
-      <c r="X60" s="14" t="n">
+      <c r="X60" s="29" t="n">
         <v>46327</v>
       </c>
       <c r="Y60" s="12" t="inlineStr"/>
@@ -14428,7 +14511,7 @@
       </c>
       <c r="V61" s="13" t="inlineStr"/>
       <c r="W61" s="13" t="inlineStr"/>
-      <c r="X61" s="18" t="n">
+      <c r="X61" s="31" t="n">
         <v>46328</v>
       </c>
       <c r="Y61" s="13" t="inlineStr"/>
@@ -14559,7 +14642,7 @@
       </c>
       <c r="V62" s="12" t="inlineStr"/>
       <c r="W62" s="12" t="inlineStr"/>
-      <c r="X62" s="14" t="n">
+      <c r="X62" s="29" t="n">
         <v>46329</v>
       </c>
       <c r="Y62" s="12" t="inlineStr"/>
@@ -14690,7 +14773,7 @@
       </c>
       <c r="V63" s="13" t="inlineStr"/>
       <c r="W63" s="13" t="inlineStr"/>
-      <c r="X63" s="18" t="n">
+      <c r="X63" s="31" t="n">
         <v>46330</v>
       </c>
       <c r="Y63" s="13" t="inlineStr"/>
@@ -14823,12 +14906,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$E:$E,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="28" t="n"/>
     </row>
     <row r="6" ht="55" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
@@ -14840,12 +14923,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$F:$F,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="27" t="n"/>
+      <c r="E6" s="27" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+      <c r="H6" s="28" t="n"/>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
@@ -14857,12 +14940,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$G:$G,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+      <c r="H7" s="28" t="n"/>
     </row>
     <row r="8" ht="55" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
@@ -14874,12 +14957,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$H:$H,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="28" t="n"/>
     </row>
     <row r="9" ht="55" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
@@ -14888,12 +14971,12 @@
         </is>
       </c>
       <c r="B9" s="25" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="C9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="33" t="n"/>
+      <c r="F9" s="33" t="n"/>
+      <c r="G9" s="33" t="n"/>
+      <c r="H9" s="34" t="n"/>
     </row>
     <row r="10" ht="55" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
@@ -14902,12 +14985,12 @@
         </is>
       </c>
       <c r="B10" s="25" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="33" t="n"/>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="34" t="n"/>
     </row>
     <row r="11" ht="55" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
@@ -14916,12 +14999,12 @@
         </is>
       </c>
       <c r="B11" s="25" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="33" t="n"/>
+      <c r="F11" s="33" t="n"/>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="34" t="n"/>
     </row>
     <row r="12" ht="55" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
@@ -14933,12 +15016,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$K:$K,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="C12" s="27" t="n"/>
+      <c r="D12" s="27" t="n"/>
+      <c r="E12" s="27" t="n"/>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+      <c r="H12" s="28" t="n"/>
     </row>
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
@@ -14950,12 +15033,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$M:$M,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+      <c r="H13" s="28" t="n"/>
     </row>
     <row r="14" ht="55" customHeight="1">
       <c r="A14" s="24" t="inlineStr">
@@ -14967,12 +15050,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$O:$O,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="28" t="n"/>
     </row>
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="24" t="inlineStr">
@@ -14984,12 +15067,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$P:$P,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="27" t="n"/>
+      <c r="E15" s="27" t="n"/>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="28" t="n"/>
     </row>
     <row r="16" ht="100" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
@@ -15001,12 +15084,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$Q:$Q,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="28" t="n"/>
     </row>
     <row r="17" ht="55" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
@@ -15018,12 +15101,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$R:$R,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
+      <c r="C17" s="27" t="n"/>
+      <c r="D17" s="27" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="28" t="n"/>
     </row>
     <row r="18" ht="55" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
@@ -15035,12 +15118,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$S:$S,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="28" t="n"/>
     </row>
     <row r="19" ht="55" customHeight="1">
       <c r="A19" s="24" t="inlineStr">
@@ -15052,12 +15135,12 @@
         <f>IFERROR(INDEX('تقویم محتوا'!$T:$T,MATCH($B$3,'تقویم محتوا'!$A:$A,0)),"")</f>
         <v/>
       </c>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="28" t="n"/>
     </row>
     <row r="20" ht="55" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
@@ -15066,12 +15149,12 @@
         </is>
       </c>
       <c r="B20" s="25" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="33" t="n"/>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="34" t="n"/>
     </row>
     <row r="21" ht="100" customHeight="1">
       <c r="A21" s="24" t="inlineStr">
@@ -15080,12 +15163,12 @@
         </is>
       </c>
       <c r="B21" s="25" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="34" t="n"/>
     </row>
     <row r="22" ht="55" customHeight="1">
       <c r="A22" s="24" t="inlineStr">
@@ -15094,12 +15177,12 @@
         </is>
       </c>
       <c r="B22" s="25" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="33" t="n"/>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="34" t="n"/>
     </row>
     <row r="23" ht="55" customHeight="1">
       <c r="A23" s="24" t="inlineStr">
@@ -15108,12 +15191,12 @@
         </is>
       </c>
       <c r="B23" s="25" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="34" t="n"/>
     </row>
     <row r="24" ht="55" customHeight="1">
       <c r="A24" s="24" t="inlineStr">
@@ -15122,12 +15205,12 @@
         </is>
       </c>
       <c r="B24" s="25" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="33" t="n"/>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="34" t="n"/>
     </row>
     <row r="25" ht="100" customHeight="1">
       <c r="A25" s="24" t="inlineStr">
@@ -15136,12 +15219,12 @@
         </is>
       </c>
       <c r="B25" s="25" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="33" t="n"/>
+      <c r="E25" s="33" t="n"/>
+      <c r="F25" s="33" t="n"/>
+      <c r="G25" s="33" t="n"/>
+      <c r="H25" s="34" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="23">

</xml_diff>